<commit_message>
Add Top-25 vendor contact directory (page + spreadsheet tab)
New 'Contacts (Top 25)' sheet in the workbook and a standalone filterable
contact-directory web page for the 25 top-ranked vendors: official website,
HQ, how-to-reach route, public phone where listed, LinkedIn company page,
and focus. Corrected domains verified via research (e.g., Bond = bondbl.com,
Loyalty Juggernaut = lji.io). Personal emails and direct dials intentionally
omitted to avoid inaccurate data.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BSASdSR9JaDPirQ4gmHWTu
</commit_message>
<xml_diff>
--- a/loyalty-software-vendors-comparison.xlsx
+++ b/loyalty-software-vendors-comparison.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Loyalty Vendor Comparison" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legend &amp; Methodology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Contacts (Top 25)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Loyalty Vendor Comparison'!$A$1:$R$151</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +71,18 @@
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002C3690"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="006B7288"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -115,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -152,6 +165,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14454,4 +14476,1044 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>How to reach</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Phone (public)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn company page</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Epsilon</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>epsilon.com</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Irving, TX, USA</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Contact form on site — ask for Loyalty/CRM (PeopleCloud) sales</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/epsilon</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty + data cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Capillary Technologies</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>capillarytech.com</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Bengaluru, IN / Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>'Contact us' / request demo — enterprise RFP</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/capillary-technologies</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty + engagement AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Comarch</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>comarch.com</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Kraków, Poland</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>'Contact' — Loyalty &amp; Marketing business unit</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/comarch</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Oracle (CrowdTwist)</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>oracle.com/cx/marketing/loyalty</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Austin, TX, USA</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Via Oracle CX / Advertising &amp; CX sales</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/oracle</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty within Oracle CX</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Salesforce Loyalty Mgmt</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>salesforce.com/products/loyalty-management</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Via your Salesforce account exec / contact form</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>1-800-664-9073</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/salesforce</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>CRM-native loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>SAP Emarsys</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>emarsys.com</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Vienna, AT / London, UK</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>'Request a demo' form</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/emarsys</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Omnichannel marketing + loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Marigold (Cheetah)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>meetmarigold.com</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Nashville / Atlanta, USA</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>meetmarigold.com/contact-sales</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/meet-marigold</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty + messaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Kobie Marketing</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>kobie.com</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>St. Petersburg, FL, USA</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>kobie.com/contact</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/kobie-marketing</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Managed enterprise loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Antavo</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>antavo.com</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>London, UK / Budapest, HU</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>antavo.com/book-demo (or /contact)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/antavo</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>No-code enterprise loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Bond Brand Loyalty</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>bondbl.com</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Toronto, ON, Canada</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>'Contact' on bondbl.com — agency/strategy</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/bond-brand-loyalty</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty agency + platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Kognitiv (Aimia)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>kognitiv.com</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Toronto, ON, Canada</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>kognitiv.com — 'Contact us'</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/kognitiv-corporation</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty + AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Merkle</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>merkle.com</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Columbia, MD, USA</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>merkle.com/contact-us — Dentsu agency</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/merkle</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty agency + tech</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Brierley</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>brierley.com</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Frisco, TX, USA</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>brierley.com/contact</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>+1 214-743-5454</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/brierley-and-partners</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Managed enterprise loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Annex Cloud</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>annexcloud.com</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Agoura Hills, CA, USA</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>annexcloud.com/contact-us</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/annex-cloud</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty experience platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Mastercard (SessionM)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>mastercard.com</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Purchase, NY, USA</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Via Mastercard Services / Loyalty sales</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/mastercard</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty + data</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Loyalty Juggernaut</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>lji.io</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Milpitas, CA, USA</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>lji.io — 'Contact' / GRAVTY demo</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/loyalty-juggernaut</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Cloud-native enterprise loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty Prime</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>loyaltyprime.com</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>loyaltyprime.com/en — 'Contact' (verify current status)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/loyalty-prime</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise loyalty platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Zinrelo</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>zinrelo.com</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>San Jose, CA, USA</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>zinrelo.com — 'Contact us' / demo</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>+1 650-701-7759</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/zinrelo</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Mid-market loyalty SaaS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Ansira</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>ansira.com</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>St. Louis, MO, USA</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>ansira.com/contact — distributed/channel</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/ansira</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Distributed marketing + loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>ICF Next</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>icf.com/next</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Reston, VA, USA</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>icf.com/contact-us</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/icf</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty consultancy + platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Maritz Motivation</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>maritzmotivation.com</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Fenton, MO, USA</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>maritzmotivation.com — 'Contact us'</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/maritz</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Loyalty &amp; incentive solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Collinson</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>collinsongroup.com</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>collinsongroup.com — 'Contact us'</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/collinson</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Loyalty + travel benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Splio</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>splio.com</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>splio.com — 'Contact' (EU)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/splio</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Individuation marketing + loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Eagle Eye Solutions</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>eagleeye.com</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Guildford, UK</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>eagleeye.com/contact</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/eagle-eye-solutions</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Real-time loyalty + promotions</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Talon.One</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>talon.one</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>talon.one/request-demo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/talon-one</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>API-first promotion + loyalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Note: Emails and direct-dial numbers are intentionally omitted to avoid inaccurate data. Reach vendors via the website contact/demo route or LinkedIn; phone shown only where publicly listed. For named decision-makers with verified emails, enrich via Apollo.io / Clay.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B28:H28"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId50"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>